<commit_message>
append elements not in official list
</commit_message>
<xml_diff>
--- a/data/matches.xlsx
+++ b/data/matches.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y34"/>
+  <dimension ref="A1:Z35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,126 +362,131 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>SortID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ATOM-ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Wissenschaftlicher Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Deutscher Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RL 2020</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>RL 2010</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NRTL 2020</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>NRTL 2010</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>NRBU 2020</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>NRBU 2010</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>WB/_x000D_
 WT 2020</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>WB/_x000D_
 WT 2010</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>WEBL 2020</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>WEBL 2010</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>EI/_x000D_
 SG 2020</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>EI/_x000D_
 SG 2010</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>SÜBL 2020</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>SÜBL 2010</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>BRG 2020</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>BRG 2010</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Neo-biota</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>§_x000D_
 Verant._x000D_
 End</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Anm. 1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Anm. 2</t>
         </is>
@@ -491,29 +496,24 @@
       <c r="A2" t="b">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>111</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>1341</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Anthoxanthum odoratum</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Gewöhnliches Ruchgras</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>*</t>
@@ -585,6 +585,11 @@
         </is>
       </c>
       <c r="U2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -594,29 +599,24 @@
       <c r="A3" t="b">
         <v>0</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>28</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>147319</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Agrostis capillaris</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Rotes Straußgras</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>*</t>
@@ -688,6 +688,11 @@
         </is>
       </c>
       <c r="U3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -697,29 +702,24 @@
       <c r="A4" t="b">
         <v>0</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>255</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>1598</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Calluna vulgaris</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Heidekraut</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>*</t>
@@ -727,14 +727,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>*</t>
@@ -787,10 +787,15 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -800,29 +805,24 @@
       <c r="A5" t="b">
         <v>0</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>690</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>147562</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Filago minima</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Zwerg-Filzkraut</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>*</t>
@@ -830,14 +830,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>*</t>
@@ -850,50 +850,55 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -903,29 +908,24 @@
       <c r="A6" t="b">
         <v>0</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>1014</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>147810</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Hieracium pilosella</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Mausohr-Habichtskraut</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>*</t>
@@ -997,6 +997,11 @@
         </is>
       </c>
       <c r="U6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1006,29 +1011,24 @@
       <c r="A7" t="b">
         <v>1</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>1106</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>168634</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Hypericum perforatum subsp. perforatum</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Tüpfel-Johanniskraut</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>*</t>
@@ -1100,6 +1100,11 @@
         </is>
       </c>
       <c r="U7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1109,29 +1114,24 @@
       <c r="A8" t="b">
         <v>0</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>1111</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>147876</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Hypochaeris radicata</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Gewöhnliches Ferkelkraut</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>*</t>
@@ -1203,6 +1203,11 @@
         </is>
       </c>
       <c r="U8" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1212,54 +1217,49 @@
       <c r="A9" t="b">
         <v>0</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>1240</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>2821</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Lotus corniculatus</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Gewöhnlicher Hornklee</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>V</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>*</t>
@@ -1302,20 +1302,25 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>R, K</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>Ansaatsippen von L. corniculatus var. sativus verdrängen zunehmend die heimische Sippe (Mause);</t>
         </is>
@@ -1325,29 +1330,24 @@
       <c r="A10" t="b">
         <v>0</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>1399</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>148240</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Ornithopus perpusillus</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Kleiner Vogelfuß</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>*</t>
@@ -1385,40 +1385,45 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -1428,29 +1433,24 @@
       <c r="A11" t="b">
         <v>1</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>1899</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>3761</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Rumex acetosella subsp. acetosella</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Kleiner Sauerampfer</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>*</t>
@@ -1522,6 +1522,11 @@
         </is>
       </c>
       <c r="U11" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1531,100 +1536,100 @@
       <c r="A12" t="b">
         <v>0</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>744</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>147652</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Genista anglica</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Englischer Ginster</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>1S</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>1S</t>
         </is>
@@ -1634,29 +1639,24 @@
       <c r="A13" t="b">
         <v>0</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>2232</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>4344</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Veronica officinalis</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Wald-Ehrenpreis</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>*</t>
@@ -1728,6 +1728,11 @@
         </is>
       </c>
       <c r="U13" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1737,29 +1742,24 @@
       <c r="A14" t="b">
         <v>1</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>57</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>164039</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Alisma plantago-aquatica s.str.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Gewöhnlicher Froschlöffel</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>*</t>
@@ -1835,7 +1835,12 @@
           <t>*</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1845,44 +1850,39 @@
       <c r="A15" t="b">
         <v>0</v>
       </c>
-      <c r="B15">
+      <c r="C15">
         <v>295</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>1670</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Carex demissa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Aufsteigende Gelb-Segge</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>*</t>
@@ -1935,15 +1935,20 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>SÜBL: Rückläufig im nördlichen Bergischen Land (Sonnenburg);</t>
         </is>
@@ -1953,29 +1958,24 @@
       <c r="A16" t="b">
         <v>0</v>
       </c>
-      <c r="B16">
+      <c r="C16">
         <v>315</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>1699</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Carex leporina</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Hasenpfoten-Segge</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>*</t>
@@ -2003,14 +2003,14 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>*</t>
@@ -2047,6 +2047,11 @@
         </is>
       </c>
       <c r="U16" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2056,105 +2061,105 @@
       <c r="A17" t="b">
         <v>0</v>
       </c>
-      <c r="B17">
+      <c r="C17">
         <v>324</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>1714</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Carex panicea</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Hirse-Segge</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>*S</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>BRG: Vorkommen im Ballungsraum erloschen (Keil);</t>
         </is>
@@ -2164,105 +2169,105 @@
       <c r="A18" t="b">
         <v>0</v>
       </c>
-      <c r="B18">
+      <c r="C18">
         <v>542</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>147428</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Drosera intermedia</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Mittlerer Sonnentau</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>2S</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>2S</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>2S</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>2S</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>§</t>
         </is>
@@ -2272,29 +2277,24 @@
       <c r="A19" t="b">
         <v>0</v>
       </c>
-      <c r="B19">
+      <c r="C19">
         <v>575</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>147467</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Eleocharis vulgaris</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Gewöhnliche Sumpfbinse</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>*</t>
@@ -2366,6 +2366,11 @@
         </is>
       </c>
       <c r="U19" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2375,29 +2380,24 @@
       <c r="A20" t="b">
         <v>0</v>
       </c>
-      <c r="B20">
+      <c r="C20">
         <v>607</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>147513</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Equisetum arvense</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Acker-Schachtelhalm</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>*</t>
@@ -2469,6 +2469,11 @@
         </is>
       </c>
       <c r="U20" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2478,29 +2483,24 @@
       <c r="A21" t="b">
         <v>0</v>
       </c>
-      <c r="B21">
+      <c r="C21">
         <v>732</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>147632</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Galium palustre</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Sumpf-Labkraut</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>*</t>
@@ -2572,6 +2572,11 @@
         </is>
       </c>
       <c r="U21" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2581,29 +2586,24 @@
       <c r="A22" t="b">
         <v>0</v>
       </c>
-      <c r="B22">
+      <c r="C22">
         <v>1134</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>147918</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Juncus articulatus</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Glieder-Binse</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>*</t>
@@ -2675,6 +2675,11 @@
         </is>
       </c>
       <c r="U22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2684,29 +2689,24 @@
       <c r="A23" t="b">
         <v>1</v>
       </c>
-      <c r="B23">
+      <c r="C23">
         <v>1135</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>147921</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Juncus bufonius s.str.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Kröten-Binse</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>*</t>
@@ -2778,6 +2778,11 @@
         </is>
       </c>
       <c r="U23" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2787,29 +2792,24 @@
       <c r="A24" t="b">
         <v>0</v>
       </c>
-      <c r="B24">
+      <c r="C24">
         <v>1139</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>147929</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Juncus conglomeratus</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Knäuel-Binse</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>*</t>
@@ -2881,6 +2881,11 @@
         </is>
       </c>
       <c r="U24" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2890,29 +2895,24 @@
       <c r="A25" t="b">
         <v>1</v>
       </c>
-      <c r="B25">
+      <c r="C25">
         <v>1262</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>168653</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Lycopus europaeus subsp. europaeus</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Ufer-Wolfstrapp</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>*</t>
@@ -2984,6 +2984,11 @@
         </is>
       </c>
       <c r="U25" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -2993,29 +2998,24 @@
       <c r="A26" t="b">
         <v>0</v>
       </c>
-      <c r="B26">
+      <c r="C26">
         <v>1242</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>2824</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Lotus pedunculatus</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Sumpf-Hornklee</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>*</t>
@@ -3091,7 +3091,12 @@
           <t>*</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
         <is>
           <t>U</t>
         </is>
@@ -3101,29 +3106,24 @@
       <c r="A27" t="b">
         <v>0</v>
       </c>
-      <c r="B27">
+      <c r="C27">
         <v>1265</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>2855</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Lysimachia nummularia</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Pfennigkraut</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>*</t>
@@ -3195,6 +3195,11 @@
         </is>
       </c>
       <c r="U27" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -3204,29 +3209,24 @@
       <c r="A28" t="b">
         <v>0</v>
       </c>
-      <c r="B28">
+      <c r="C28">
         <v>1268</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>2858</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Lysimachia vulgaris</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Gewöhnlicher Gilbweiderich</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>*</t>
@@ -3298,6 +3298,11 @@
         </is>
       </c>
       <c r="U28" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -3307,29 +3312,24 @@
       <c r="A29" t="b">
         <v>0</v>
       </c>
-      <c r="B29">
+      <c r="C29">
         <v>1270</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>2860</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Lythrum salicaria</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Blut-Weiderich</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>*</t>
@@ -3405,7 +3405,12 @@
           <t>*</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3415,29 +3420,24 @@
       <c r="A30" t="b">
         <v>0</v>
       </c>
-      <c r="B30">
+      <c r="C30">
         <v>1440</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>148312</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Peplis portula</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Sumpfquendel</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>*</t>
@@ -3445,19 +3445,19 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>*</t>
@@ -3465,29 +3465,29 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="Q30" t="inlineStr">
         <is>
           <t>*</t>
@@ -3505,10 +3505,15 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3518,39 +3523,34 @@
       <c r="A31" t="b">
         <v>0</v>
       </c>
-      <c r="B31">
+      <c r="C31">
         <v>1617</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>3467</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Ranunculus flammula</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Brennender Hahnenfuß</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>*</t>
@@ -3612,6 +3612,11 @@
         </is>
       </c>
       <c r="U31" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -3621,100 +3626,100 @@
       <c r="A32" t="b">
         <v>0</v>
       </c>
-      <c r="B32">
+      <c r="C32">
         <v>2090</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>4084</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Stellaria palustris</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Sumpf-Sternmiere</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="R32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="S32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -3724,29 +3729,24 @@
       <c r="A33" t="b">
         <v>1</v>
       </c>
-      <c r="B33">
+      <c r="C33">
         <v>2222</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>167277</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Veronica anagallis-aquatica s.str.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Blauer Wasser-Ehrenpreis</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>*</t>
@@ -3814,10 +3814,15 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="V33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3827,102 +3832,112 @@
       <c r="A34" t="b">
         <v>0</v>
       </c>
-      <c r="B34">
+      <c r="C34">
         <v>2238</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>4352</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Veronica scutellata</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Schild-Ehrenpreis</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="R34" t="inlineStr">
         <is>
           <t>3S</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
+      <c r="S34" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
+      <c r="T34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="U34" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="V34" t="inlineStr">
         <is>
           <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Festuca ovina</t>
         </is>
       </c>
     </row>

</xml_diff>